<commit_message>
Update Day 3 activity data~
</commit_message>
<xml_diff>
--- a/data/12616002.xlsx
+++ b/data/12616002.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CAP776\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30FCDB4-B002-4C88-BCA0-B96D1807ACC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DB1E695-74D9-4402-B1ED-D2A019807C70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="41">
   <si>
     <t>My Data, My Story</t>
   </si>
@@ -174,6 +174,12 @@
   </si>
   <si>
     <t>2026-08-22</t>
+  </si>
+  <si>
+    <t>2026-08-23</t>
+  </si>
+  <si>
+    <t>High productivity</t>
   </si>
 </sst>
 </file>
@@ -819,23 +825,50 @@
       </c>
     </row>
     <row r="8" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="5" t="str">
+      <c r="A8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="4">
+        <v>539</v>
+      </c>
+      <c r="C8" s="13">
+        <v>40</v>
+      </c>
+      <c r="D8" s="13">
+        <v>94</v>
+      </c>
+      <c r="E8" s="13">
+        <v>107</v>
+      </c>
+      <c r="F8" s="13">
+        <v>0</v>
+      </c>
+      <c r="G8" s="13">
+        <v>0</v>
+      </c>
+      <c r="H8" s="13">
+        <v>260</v>
+      </c>
+      <c r="I8" s="5">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J8" s="5"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="6"/>
+        <v>1040</v>
+      </c>
+      <c r="J8" s="5">
+        <f t="shared" ref="J8:J9" si="1">IF(I8="","",1440-I8)</f>
+        <v>400</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="6" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="9" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3"/>
@@ -850,7 +883,10 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J9" s="5"/>
+      <c r="J9" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>

</xml_diff>